<commit_message>
fix accesos de usuarios y permisos, correcion de plantillas
</commit_message>
<xml_diff>
--- a/backend/app/templates/excel/plantilla_de_sueldos_y_salarios.xlsx
+++ b/backend/app/templates/excel/plantilla_de_sueldos_y_salarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\sistema_de_boletas_de_pago-RengifoLtda\backend\app\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{284A849A-FDFD-4FD1-8E35-B13857E9491C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B93374-F68B-4BA3-9948-F641908D956C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4AB49BEC-9586-4F07-8E7B-5982E757BCB2}"/>
   </bookViews>
@@ -155,20 +155,20 @@
     <t>FIRMA</t>
   </si>
   <si>
-    <t>…............................................................................................................................................................</t>
-  </si>
-  <si>
-    <t>…..........................................................................................................</t>
-  </si>
-  <si>
-    <t>….................................................................................................</t>
+    <t>…........................................................................................................................</t>
+  </si>
+  <si>
+    <t>…..........................................................................</t>
+  </si>
+  <si>
+    <t>….......................................................................</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -222,6 +222,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -328,7 +336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -339,9 +347,30 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -351,23 +380,17 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -384,11 +407,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -399,18 +419,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -748,7 +757,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X17"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" customWidth="1"/>
@@ -776,7 +785,7 @@
     <col min="24" max="24" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -802,65 +811,65 @@
       <c r="W1" s="3"/>
       <c r="X1" s="3"/>
     </row>
-    <row r="2" spans="1:24" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:27" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="7"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="14"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="9" t="s">
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="10"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
-      <c r="U2" s="11" t="s">
+      <c r="U2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="V2" s="12"/>
-      <c r="W2" s="11" t="s">
+      <c r="V2" s="6"/>
+      <c r="W2" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="X2" s="12"/>
-    </row>
-    <row r="3" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="X2" s="6"/>
+    </row>
+    <row r="3" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="7"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="14"/>
       <c r="K3" s="3"/>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
@@ -868,7 +877,7 @@
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
     </row>
-    <row r="4" spans="1:24" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -894,7 +903,7 @@
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
     </row>
-    <row r="5" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -904,14 +913,14 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
@@ -922,7 +931,7 @@
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -932,27 +941,27 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="18" t="s">
+      <c r="J6" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="1"/>
-      <c r="U6" s="14" t="s">
+      <c r="S6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="V6" s="15"/>
-      <c r="W6" s="15"/>
-      <c r="X6" s="15"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
+      <c r="X6" s="19"/>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -978,217 +987,218 @@
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
     </row>
-    <row r="8" spans="1:24" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+    <row r="8" spans="1:27" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="J8" s="19" t="s">
+      <c r="J8" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="K8" s="19" t="s">
+      <c r="K8" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="19" t="s">
+      <c r="L8" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="M8" s="19" t="s">
+      <c r="M8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="N8" s="19" t="s">
+      <c r="N8" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="O8" s="19" t="s">
+      <c r="O8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="P8" s="19" t="s">
+      <c r="P8" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="19" t="s">
+      <c r="Q8" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="R8" s="19" t="s">
+      <c r="R8" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="S8" s="19" t="s">
+      <c r="S8" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="T8" s="19" t="s">
+      <c r="T8" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="U8" s="19" t="s">
+      <c r="U8" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="V8" s="19" t="s">
+      <c r="V8" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="W8" s="19" t="s">
+      <c r="W8" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="X8" s="19" t="s">
+      <c r="X8" s="15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="19"/>
-      <c r="T9" s="19"/>
-      <c r="U9" s="19"/>
-      <c r="V9" s="19"/>
-      <c r="W9" s="19"/>
-      <c r="X9" s="19"/>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="19"/>
-      <c r="P10" s="19"/>
-      <c r="Q10" s="19"/>
-      <c r="R10" s="19"/>
-      <c r="S10" s="19"/>
-      <c r="T10" s="19"/>
-      <c r="U10" s="19"/>
-      <c r="V10" s="19"/>
-      <c r="W10" s="19"/>
-      <c r="X10" s="19"/>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A11" s="20">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="15"/>
+      <c r="S9" s="15"/>
+      <c r="T9" s="15"/>
+      <c r="U9" s="15"/>
+      <c r="V9" s="15"/>
+      <c r="W9" s="15"/>
+      <c r="X9" s="15"/>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="15"/>
+      <c r="T10" s="15"/>
+      <c r="U10" s="15"/>
+      <c r="V10" s="15"/>
+      <c r="W10" s="15"/>
+      <c r="X10" s="15"/>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" s="7">
         <v>1</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
-      <c r="O11" s="20"/>
-      <c r="P11" s="20"/>
-      <c r="Q11" s="20"/>
-      <c r="R11" s="20"/>
-      <c r="S11" s="20"/>
-      <c r="T11" s="20"/>
-      <c r="U11" s="20"/>
-      <c r="V11" s="20"/>
-      <c r="W11" s="20"/>
-      <c r="X11" s="20"/>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="20">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="7"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="7"/>
+      <c r="T11" s="7"/>
+      <c r="U11" s="7"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="7"/>
+      <c r="X11" s="7"/>
+      <c r="AA11" s="28"/>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
         <v>2</v>
       </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
-      <c r="M12" s="20"/>
-      <c r="N12" s="20"/>
-      <c r="O12" s="20"/>
-      <c r="P12" s="20"/>
-      <c r="Q12" s="20"/>
-      <c r="R12" s="20"/>
-      <c r="S12" s="20"/>
-      <c r="T12" s="20"/>
-      <c r="U12" s="20"/>
-      <c r="V12" s="20"/>
-      <c r="W12" s="20"/>
-      <c r="X12" s="20"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7"/>
+      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="7"/>
+      <c r="V12" s="7"/>
+      <c r="W12" s="7"/>
+      <c r="X12" s="7"/>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="24"/>
-      <c r="L13" s="24"/>
-      <c r="M13" s="24"/>
-      <c r="N13" s="24"/>
-      <c r="O13" s="24"/>
-      <c r="P13" s="24"/>
-      <c r="Q13" s="24"/>
-      <c r="R13" s="24"/>
-      <c r="S13" s="24"/>
-      <c r="T13" s="24"/>
-      <c r="U13" s="24"/>
-      <c r="V13" s="24"/>
-      <c r="W13" s="24"/>
-      <c r="X13" s="24"/>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1214,7 +1224,7 @@
       <c r="W14" s="1"/>
       <c r="X14" s="1"/>
     </row>
-    <row r="15" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1240,34 +1250,34 @@
       <c r="W15" s="1"/>
       <c r="X15" s="1"/>
     </row>
-    <row r="16" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
-      <c r="L16" s="25" t="s">
+      <c r="L16" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="M16" s="25"/>
-      <c r="N16" s="25"/>
-      <c r="O16" s="25"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+      <c r="O16" s="24"/>
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
-      <c r="R16" s="25" t="s">
+      <c r="R16" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="S16" s="25"/>
-      <c r="T16" s="25"/>
-      <c r="U16" s="25"/>
+      <c r="S16" s="24"/>
+      <c r="T16" s="24"/>
+      <c r="U16" s="24"/>
       <c r="V16" s="1"/>
       <c r="W16" s="1"/>
       <c r="X16" s="1"/>
@@ -1276,62 +1286,46 @@
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
-      <c r="L17" s="14" t="s">
+      <c r="L17" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="M17" s="15"/>
-      <c r="N17" s="15"/>
-      <c r="O17" s="15"/>
+      <c r="M17" s="20"/>
+      <c r="N17" s="20"/>
+      <c r="O17" s="20"/>
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
-      <c r="R17" s="26" t="s">
+      <c r="R17" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="S17" s="27"/>
-      <c r="T17" s="27"/>
-      <c r="U17" s="27"/>
+      <c r="S17" s="18"/>
+      <c r="T17" s="18"/>
+      <c r="U17" s="18"/>
       <c r="V17" s="1"/>
       <c r="W17" s="1"/>
       <c r="X17" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="P3:R3"/>
-    <mergeCell ref="L3:O3"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="D2:J2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="S8:S10"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="N8:N10"/>
-    <mergeCell ref="O8:O10"/>
-    <mergeCell ref="P8:P10"/>
-    <mergeCell ref="Q8:Q10"/>
-    <mergeCell ref="R8:R10"/>
-    <mergeCell ref="G8:G10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="R16:U16"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="D17:I17"/>
+    <mergeCell ref="D16:I16"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="L16:O16"/>
+    <mergeCell ref="S6:X6"/>
     <mergeCell ref="R17:U17"/>
-    <mergeCell ref="U6:X6"/>
     <mergeCell ref="J5:O5"/>
     <mergeCell ref="J6:O6"/>
     <mergeCell ref="T8:T10"/>
@@ -1340,14 +1334,30 @@
     <mergeCell ref="W8:W10"/>
     <mergeCell ref="X8:X10"/>
     <mergeCell ref="L8:L10"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="R16:U16"/>
-    <mergeCell ref="P2:R2"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="D17:I17"/>
-    <mergeCell ref="D16:I16"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="L16:O16"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="S8:S10"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="N8:N10"/>
+    <mergeCell ref="O8:O10"/>
+    <mergeCell ref="P8:P10"/>
+    <mergeCell ref="Q8:Q10"/>
+    <mergeCell ref="R8:R10"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="L3:O3"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="D2:J2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.74803149606299213" bottom="0.19685039370078741" header="0.19685039370078741" footer="0.19685039370078741"/>
   <pageSetup scale="44" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix plantillas de exportacion y estandarizacion
</commit_message>
<xml_diff>
--- a/backend/app/templates/excel/plantilla_de_sueldos_y_salarios.xlsx
+++ b/backend/app/templates/excel/plantilla_de_sueldos_y_salarios.xlsx
@@ -115,7 +115,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -260,11 +260,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -392,6 +398,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1098,7 +1107,8 @@
       </c>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>Gestora Pública de Bolivia</t>
+          <t>Aportes Gestora Pública
+12.71%</t>
         </is>
       </c>
       <c r="T8" s="10" t="inlineStr">
@@ -1322,7 +1332,7 @@
       <c r="A16" s="1" t="n"/>
       <c r="B16" s="1" t="n"/>
       <c r="C16" s="1" t="n"/>
-      <c r="D16" s="40" t="n"/>
+      <c r="D16" s="49" t="n"/>
       <c r="E16" s="48" t="n"/>
       <c r="F16" s="48" t="n"/>
       <c r="G16" s="48" t="n"/>
@@ -1330,13 +1340,13 @@
       <c r="I16" s="48" t="n"/>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
-      <c r="L16" s="40" t="n"/>
+      <c r="L16" s="49" t="n"/>
       <c r="M16" s="48" t="n"/>
       <c r="N16" s="48" t="n"/>
       <c r="O16" s="48" t="n"/>
       <c r="P16" s="2" t="n"/>
       <c r="Q16" s="2" t="n"/>
-      <c r="R16" s="40" t="n"/>
+      <c r="R16" s="49" t="n"/>
       <c r="S16" s="48" t="n"/>
       <c r="T16" s="48" t="n"/>
       <c r="U16" s="48" t="n"/>

</xml_diff>